<commit_message>
LV_TMTT0012117_TMTT0012119 changes July 23 24
</commit_message>
<xml_diff>
--- a/TestData/TMTT0012113_ValidateCoExistFieldForGCATracking.xlsx
+++ b/TestData/TMTT0012113_ValidateCoExistFieldForGCATracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E39CF52C-6F69-4558-8CB0-604350A4193A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DF49373-E02A-4AAB-B292-E8AD115B82FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{6914B0A7-23C8-4C59-8A71-D12BF5352AB3}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{6914B0A7-23C8-4C59-8A71-D12BF5352AB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="3" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="ModuleName" sheetId="5" r:id="rId3"/>
     <sheet name="AddOpportunity" sheetId="1" r:id="rId4"/>
     <sheet name="AddContact" sheetId="2" r:id="rId5"/>
-    <sheet name="InternalTeam" sheetId="6" r:id="rId6"/>
+    <sheet name="OppDealTeamMembers" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="91">
   <si>
     <t>Client</t>
   </si>
@@ -311,6 +311,9 @@
   </si>
   <si>
     <t>Activism Advisory</t>
+  </si>
+  <si>
+    <t>Analyst</t>
   </si>
 </sst>
 </file>
@@ -354,7 +357,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -362,7 +365,6 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -698,14 +700,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{533E536B-B7DF-4CA3-886D-7CBD31363DCD}">
   <dimension ref="A1:AB4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>68</v>
       </c>
@@ -716,7 +718,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>75</v>
       </c>
@@ -733,7 +735,7 @@
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -744,7 +746,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>73</v>
       </c>
@@ -763,14 +765,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DA9484C-3321-40A2-8DBC-82467259E8DC}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -783,22 +785,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10B4AA16-114A-488D-B988-48E1BF5E1B86}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>81</v>
       </c>
@@ -811,36 +813,36 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28710558-C34E-4463-B41D-5BFD4F346D1C}">
   <dimension ref="A1:AE3"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="8.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="8.28515625" style="4" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="21" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="29.88671875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.33203125" customWidth="1"/>
-    <col min="27" max="27" width="11.44140625" customWidth="1"/>
-    <col min="29" max="29" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="29.85546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.28515625" customWidth="1"/>
+    <col min="27" max="27" width="11.42578125" customWidth="1"/>
+    <col min="29" max="29" width="21.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -935,7 +937,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -1030,14 +1032,14 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>31</v>
       </c>
       <c r="B3" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" t="s">
         <v>89</v>
       </c>
       <c r="D3" t="s">
@@ -1133,17 +1135,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{935637E3-2FF3-414E-8DF7-082775A8C6A6}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>55</v>
       </c>
@@ -1169,7 +1171,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -1202,34 +1204,44 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50423EC6-F997-4E60-A436-3E9753BC8546}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>83</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>82</v>
       </c>
       <c r="B2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>86</v>
       </c>
       <c r="B3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" t="s">
         <v>87</v>
       </c>
     </row>

</xml_diff>